<commit_message>
added RCMI landing page
</commit_message>
<xml_diff>
--- a/workbook/rcmi_content.xlsx
+++ b/workbook/rcmi_content.xlsx
@@ -666,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO40"/>
+  <dimension ref="A1:AP41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -894,6 +894,11 @@
           <t>NCBI URL</t>
         </is>
       </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>Designation</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -1205,6 +1210,11 @@
           <t>GWW, PPP</t>
         </is>
       </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Executive Director; RIC Lead</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -1227,7 +1237,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>RCMI Leadership</t>
+          <t>Community Engagement Core</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1301,6 +1311,11 @@
           <t>Dr. Payam Sheikhattari</t>
         </is>
       </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>CEC PI</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -1323,7 +1338,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Research Staff</t>
+          <t>RCMI Leadership</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1397,6 +1412,11 @@
           <t>Diane Hughes</t>
         </is>
       </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>Program Manager</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1419,7 +1439,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1462,7 +1482,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1505,7 +1525,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1553,7 +1573,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1596,7 +1616,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1639,7 +1659,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1682,7 +1702,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1725,7 +1745,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1768,7 +1788,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1811,7 +1831,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1854,7 +1874,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1897,7 +1917,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1945,7 +1965,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1988,7 +2008,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2031,7 +2051,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2079,7 +2099,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2122,7 +2142,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2165,7 +2185,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2208,7 +2228,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2251,7 +2271,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2309,7 +2329,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2347,7 +2367,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2400,7 +2420,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2458,7 +2478,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2516,7 +2536,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2574,7 +2594,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2632,7 +2652,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2690,7 +2710,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2748,7 +2768,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2806,7 +2826,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2864,7 +2884,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2917,7 +2937,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2970,7 +2990,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Pilot Faculty</t>
+          <t>IDC Pilot Faculties</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3174,6 +3194,76 @@
       <c r="AO40" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/?term=meeker+tj</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>faculty_paul_tchounwou</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>30</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Dr. Paul B. Tchounwou</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>RCMI Leadership</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Dean, School of Computer, Mathematical and Natural Sciences</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>School of Computer, Mathematical and Natural Sciences</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Research Interests</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Environmental toxicology, health disparities research, and RCMI program leadership and administration.</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>paul.tchounwou@morgan.edu</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>./img/faculty/governance_paul_tchounwou.jpg</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>Dr. Paul B. Tchounwou</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>Dr. Paul B. Tchounwou is Dean of the School of Computer, Mathematical and Natural Sciences (SCMNS) at Morgan State University (MSU) and is responsible for oversight of the RCMI grant. In his capacity as Dean, his primary responsibilities include overseeing the academic enterprise and guiding the continued advancement of SCMNS's research, education and training programs. Prior to joining MSU, Dr. Tchounwou served as Presidential Distinguished Professor; Associate Dean for Research, Graduate Studies and International Programs in the College of Science, Engineering and Technology, and Executive Director of RCMI Center for Health Disparities Research at Jackson State University (JSU). He is credited for leading the RCMI Program at JSU for more than 15 years. Dr. Tchounwou also directed the RCMI Translational Research Network Data Coordinating Center. He has been a very active leader in the RCMI Consortium where he currently serves as Multi-PI of the RCMI Coordinating Center, providing leadership for the coordination of its Research Infrastructure Core domain. Dr. Tchounwou, who has published over 300 peer-reviewed papers in top-tier scientific journals and books, is a nationally and internationally known biomedical scientist. He is the Editor-In-Chief of International Journal of Environmental Research and Public Health (MDPI, Basel, Switzerland) and of Environmental Toxicology-An International Journal (John Wiley &amp; Sons, New York, USA). Dr. Tchounwou currently serves on the NIH Scientific and Technical Review Board for the Biomedical and Behavioral Research Facilities. He is also an ad-hoc member of the Reviewers Recognition Working Group of the NIH Center for Scientific Review Advisory Council (CSRAC).</t>
+        </is>
+      </c>
+      <c r="AP41" t="inlineStr">
+        <is>
+          <t>PI</t>
         </is>
       </c>
     </row>

</xml_diff>